<commit_message>
save 18 05 2026
</commit_message>
<xml_diff>
--- a/4 четверть_7_JavaScript_Advanced.xlsx
+++ b/4 четверть_7_JavaScript_Advanced.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Machenike\Desktop\Homework_repo\GB_Developer_Workbook\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AlexServHW\Desktop\GB_Developer_Workbook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D5A4825-CAD6-47D0-9AD5-8C5F093451E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1E99A4C-4C31-4743-9AF4-B8D4B4057F46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="14020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Название 1-3" sheetId="12" r:id="rId1"/>
@@ -19,6 +19,9 @@
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -2938,12 +2941,20 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="17" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -3169,9 +3180,9 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -3182,23 +3193,23 @@
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="8" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="9" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="8" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
@@ -3207,70 +3218,73 @@
     <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="12" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="13" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="12" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="13" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="10" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="8" fillId="10" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="10" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="8" fillId="10" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="11" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="8" fillId="11" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="11" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="8" fillId="11" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="49" fontId="7" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="13" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="13" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -3279,7 +3293,7 @@
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3880,38 +3894,38 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A2:V141"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="36" style="1" customWidth="1"/>
-    <col min="2" max="2" width="50.54296875" style="2" customWidth="1"/>
-    <col min="3" max="3" width="71.1796875" style="4" customWidth="1"/>
-    <col min="4" max="4" width="56.453125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="6.26953125" style="7" customWidth="1"/>
-    <col min="6" max="6" width="43.26953125" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="55.08984375" style="2" customWidth="1"/>
-    <col min="8" max="8" width="67.90625" style="1" customWidth="1"/>
-    <col min="9" max="9" width="64.36328125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="7.81640625" style="7" customWidth="1"/>
-    <col min="11" max="11" width="39.26953125" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="48.90625" style="1" customWidth="1"/>
-    <col min="13" max="13" width="72.6328125" style="1" customWidth="1"/>
-    <col min="14" max="14" width="43.90625" style="1" customWidth="1"/>
-    <col min="15" max="15" width="7.81640625" style="7" customWidth="1"/>
-    <col min="16" max="16" width="56.81640625" style="2" customWidth="1"/>
-    <col min="17" max="17" width="46.7265625" style="2" customWidth="1"/>
-    <col min="18" max="18" width="62.90625" style="2" customWidth="1"/>
-    <col min="19" max="19" width="49.1796875" style="1" customWidth="1"/>
-    <col min="20" max="20" width="8.7265625" style="8"/>
-    <col min="21" max="21" width="67.7265625" style="2" customWidth="1"/>
-    <col min="22" max="22" width="68.36328125" style="1" customWidth="1"/>
-    <col min="23" max="24" width="59.36328125" style="1" customWidth="1"/>
-    <col min="25" max="25" width="59.6328125" style="1" customWidth="1"/>
-    <col min="26" max="26" width="99.453125" style="1" customWidth="1"/>
-    <col min="27" max="27" width="41.26953125" style="1" customWidth="1"/>
-    <col min="28" max="16384" width="8.7265625" style="1"/>
+    <col min="2" max="2" width="50.5546875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="71.21875" style="4" customWidth="1"/>
+    <col min="4" max="4" width="56.44140625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="6.21875" style="7" customWidth="1"/>
+    <col min="6" max="6" width="43.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="55.109375" style="2" customWidth="1"/>
+    <col min="8" max="8" width="67.88671875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="64.33203125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="7.77734375" style="7" customWidth="1"/>
+    <col min="11" max="11" width="39.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="48.88671875" style="1" customWidth="1"/>
+    <col min="13" max="13" width="72.6640625" style="1" customWidth="1"/>
+    <col min="14" max="14" width="43.88671875" style="1" customWidth="1"/>
+    <col min="15" max="15" width="7.77734375" style="7" customWidth="1"/>
+    <col min="16" max="16" width="56.77734375" style="2" customWidth="1"/>
+    <col min="17" max="17" width="46.77734375" style="2" customWidth="1"/>
+    <col min="18" max="18" width="62.88671875" style="2" customWidth="1"/>
+    <col min="19" max="19" width="49.21875" style="1" customWidth="1"/>
+    <col min="20" max="20" width="8.77734375" style="8"/>
+    <col min="21" max="21" width="67.77734375" style="2" customWidth="1"/>
+    <col min="22" max="22" width="68.33203125" style="1" customWidth="1"/>
+    <col min="23" max="24" width="59.33203125" style="1" customWidth="1"/>
+    <col min="25" max="25" width="59.6640625" style="1" customWidth="1"/>
+    <col min="26" max="26" width="99.44140625" style="1" customWidth="1"/>
+    <col min="27" max="27" width="41.21875" style="1" customWidth="1"/>
+    <col min="28" max="16384" width="8.77734375" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A2" s="3"/>
       <c r="B2" s="5"/>
       <c r="C2" s="6"/>
@@ -3930,7 +3944,7 @@
       <c r="S2" s="5"/>
       <c r="U2" s="5"/>
     </row>
-    <row r="3" spans="1:22" ht="29" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:22" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -3941,37 +3955,37 @@
       <c r="U3" s="1"/>
       <c r="V3" s="2"/>
     </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A4" s="11" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:22" ht="29" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:22" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C5" s="9" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A6" s="12" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:22" ht="29" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:22" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C7" s="9" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:22" ht="58" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:22" ht="57.6" x14ac:dyDescent="0.3">
       <c r="C8" s="9" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A9" s="12" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:22" ht="29" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:22" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C10" s="9" t="s">
         <v>8</v>
       </c>
@@ -3979,17 +3993,17 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:22" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:22" ht="72" x14ac:dyDescent="0.3">
       <c r="C11" s="9" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:22" ht="58" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:22" ht="57.6" x14ac:dyDescent="0.3">
       <c r="C12" s="9" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A13" s="3"/>
       <c r="B13" s="5"/>
       <c r="C13" s="6"/>
@@ -4008,7 +4022,7 @@
       <c r="S13" s="5"/>
       <c r="U13" s="5"/>
     </row>
-    <row r="14" spans="1:22" ht="29" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:22" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>12</v>
       </c>
@@ -4019,7 +4033,7 @@
       <c r="U14" s="1"/>
       <c r="V14" s="2"/>
     </row>
-    <row r="15" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A15" s="11" t="s">
         <v>13</v>
       </c>
@@ -4030,7 +4044,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:22" ht="58" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:22" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A16" s="2"/>
       <c r="B16" s="9" t="s">
         <v>45</v>
@@ -4039,7 +4053,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="58" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B17" s="28" t="s">
         <v>138</v>
       </c>
@@ -4047,12 +4061,12 @@
         <v>19</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" s="12" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="116" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:4" ht="115.2" x14ac:dyDescent="0.3">
       <c r="B19" s="2" t="s">
         <v>111</v>
       </c>
@@ -4060,12 +4074,12 @@
         <v>16</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A20" s="10" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="21" spans="1:4" ht="58" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B21" s="9" t="s">
         <v>22</v>
       </c>
@@ -4073,7 +4087,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" s="12" t="s">
         <v>23</v>
       </c>
@@ -4081,7 +4095,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="23" spans="1:4" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:4" ht="129.6" x14ac:dyDescent="0.3">
       <c r="B23" s="2" t="s">
         <v>27</v>
       </c>
@@ -4092,7 +4106,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="24" spans="1:4" ht="87" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
       <c r="B24" s="2" t="s">
         <v>28</v>
       </c>
@@ -4103,12 +4117,12 @@
         <v>115</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" s="12" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="26" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A26" s="9"/>
       <c r="B26" s="25" t="s">
         <v>113</v>
@@ -4117,22 +4131,22 @@
         <v>31</v>
       </c>
     </row>
-    <row r="27" spans="1:4" ht="87" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
       <c r="C27" s="9" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" s="10" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="29" spans="1:4" ht="174" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:4" ht="172.8" x14ac:dyDescent="0.3">
       <c r="C29" s="9" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="30" spans="1:4" ht="116" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:4" ht="115.2" x14ac:dyDescent="0.3">
       <c r="B30" s="9" t="s">
         <v>35</v>
       </c>
@@ -4140,7 +4154,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31" s="12" t="s">
         <v>36</v>
       </c>
@@ -4148,7 +4162,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="32" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B32" s="9" t="s">
         <v>39</v>
       </c>
@@ -4156,7 +4170,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="33" spans="1:22" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:22" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
         <v>40</v>
       </c>
@@ -4164,7 +4178,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="34" spans="1:22" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:22" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
         <v>42</v>
       </c>
@@ -4178,7 +4192,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="35" spans="1:22" ht="116" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:22" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
         <v>47</v>
       </c>
@@ -4192,22 +4206,22 @@
         <v>48</v>
       </c>
     </row>
-    <row r="36" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A36" s="12" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="37" spans="1:22" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:22" ht="43.2" x14ac:dyDescent="0.3">
       <c r="C37" s="9" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="38" spans="1:22" ht="145" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:22" ht="144" x14ac:dyDescent="0.3">
       <c r="C38" s="9" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="39" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A39" s="3"/>
       <c r="B39" s="5"/>
       <c r="C39" s="6"/>
@@ -4226,7 +4240,7 @@
       <c r="S39" s="5"/>
       <c r="U39" s="5"/>
     </row>
-    <row r="40" spans="1:22" ht="29" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:22" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
         <v>12</v>
       </c>
@@ -4240,17 +4254,17 @@
       <c r="U40" s="1"/>
       <c r="V40" s="2"/>
     </row>
-    <row r="41" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A41" s="11" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="42" spans="1:22" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:22" ht="72" x14ac:dyDescent="0.3">
       <c r="C42" s="9" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="43" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A43" s="16" t="s">
         <v>59</v>
       </c>
@@ -4258,17 +4272,17 @@
         <v>62</v>
       </c>
     </row>
-    <row r="44" spans="1:22" ht="29" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:22" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C44" s="9" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="45" spans="1:22" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:22" ht="100.8" x14ac:dyDescent="0.3">
       <c r="C45" s="9" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="46" spans="1:22" ht="391.5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:22" ht="388.8" x14ac:dyDescent="0.3">
       <c r="A46" s="9" t="s">
         <v>64</v>
       </c>
@@ -4282,7 +4296,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="47" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A47" s="16" t="s">
         <v>68</v>
       </c>
@@ -4290,7 +4304,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="48" spans="1:22" ht="203" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:22" ht="201.6" x14ac:dyDescent="0.3">
       <c r="B48" s="2" t="s">
         <v>67</v>
       </c>
@@ -4298,12 +4312,12 @@
         <v>66</v>
       </c>
     </row>
-    <row r="49" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A49" s="16" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="50" spans="1:22" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:22" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B50" s="17" t="s">
         <v>72</v>
       </c>
@@ -4311,7 +4325,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="52" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A52" s="3"/>
       <c r="B52" s="5"/>
       <c r="C52" s="6"/>
@@ -4330,7 +4344,7 @@
       <c r="S52" s="5"/>
       <c r="U52" s="5"/>
     </row>
-    <row r="53" spans="1:22" ht="29" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:22" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A53" s="1" t="s">
         <v>73</v>
       </c>
@@ -4344,17 +4358,17 @@
       <c r="U53" s="1"/>
       <c r="V53" s="2"/>
     </row>
-    <row r="54" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A54" s="11" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="55" spans="1:22" ht="29" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:22" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C55" s="9" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="56" spans="1:22" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:22" ht="129.6" x14ac:dyDescent="0.3">
       <c r="B56" s="9" t="s">
         <v>82</v>
       </c>
@@ -4365,7 +4379,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="57" spans="1:22" ht="58" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:22" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A57" s="1" t="s">
         <v>85</v>
       </c>
@@ -4373,17 +4387,17 @@
         <v>84</v>
       </c>
     </row>
-    <row r="58" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A58" s="11" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="59" spans="1:22" ht="29" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:22" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C59" s="9" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="60" spans="1:22" ht="174" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:22" ht="172.8" x14ac:dyDescent="0.3">
       <c r="A60" s="1" t="s">
         <v>86</v>
       </c>
@@ -4397,7 +4411,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="61" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A61" s="11" t="s">
         <v>89</v>
       </c>
@@ -4405,12 +4419,12 @@
         <v>90</v>
       </c>
     </row>
-    <row r="62" spans="1:22" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:22" ht="72" x14ac:dyDescent="0.3">
       <c r="C62" s="9" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="63" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A63" s="11" t="s">
         <v>88</v>
       </c>
@@ -4418,12 +4432,12 @@
         <v>90</v>
       </c>
     </row>
-    <row r="64" spans="1:22" ht="29" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:22" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C64" s="9" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="65" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A65" s="3"/>
       <c r="B65" s="5"/>
       <c r="C65" s="6"/>
@@ -4442,7 +4456,7 @@
       <c r="S65" s="5"/>
       <c r="U65" s="5"/>
     </row>
-    <row r="66" spans="1:22" ht="29" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:22" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A66" s="1" t="s">
         <v>73</v>
       </c>
@@ -4456,7 +4470,7 @@
       <c r="U66" s="1"/>
       <c r="V66" s="2"/>
     </row>
-    <row r="67" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A67" s="19" t="s">
         <v>93</v>
       </c>
@@ -4464,7 +4478,7 @@
       <c r="C67" s="19"/>
       <c r="D67" s="20"/>
     </row>
-    <row r="68" spans="1:22" ht="188.5" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:22" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A68" s="21" t="s">
         <v>94</v>
       </c>
@@ -4474,7 +4488,7 @@
       </c>
       <c r="D68" s="22"/>
     </row>
-    <row r="69" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A69" s="23" t="s">
         <v>96</v>
       </c>
@@ -4482,7 +4496,7 @@
       <c r="C69" s="21"/>
       <c r="D69" s="22"/>
     </row>
-    <row r="70" spans="1:22" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:22" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A70" s="22"/>
       <c r="B70" s="21" t="s">
         <v>97</v>
@@ -4492,7 +4506,7 @@
       </c>
       <c r="D70" s="22"/>
     </row>
-    <row r="71" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A71" s="23" t="s">
         <v>99</v>
       </c>
@@ -4506,19 +4520,19 @@
         <v>102</v>
       </c>
     </row>
-    <row r="72" spans="1:22" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:22" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A72" s="22"/>
       <c r="B72" s="21" t="s">
         <v>103</v>
       </c>
-      <c r="C72" s="21" t="s">
+      <c r="C72" s="38" t="s">
         <v>104</v>
       </c>
       <c r="D72" s="21" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="73" spans="1:22" ht="58" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:22" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A73" s="22"/>
       <c r="B73" s="21"/>
       <c r="C73" s="21" t="s">
@@ -4528,7 +4542,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="74" spans="1:22" ht="29" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:22" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A74" s="22"/>
       <c r="B74" s="21"/>
       <c r="C74" s="21"/>
@@ -4536,7 +4550,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="75" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A75" s="3"/>
       <c r="B75" s="5"/>
       <c r="C75" s="6"/>
@@ -4555,7 +4569,7 @@
       <c r="S75" s="5"/>
       <c r="U75" s="5"/>
     </row>
-    <row r="76" spans="1:22" ht="29" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:22" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A76" s="1" t="s">
         <v>117</v>
       </c>
@@ -4569,17 +4583,17 @@
       <c r="U76" s="1"/>
       <c r="V76" s="2"/>
     </row>
-    <row r="77" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A77" s="11" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="78" spans="1:22" ht="58" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:22" ht="57.6" x14ac:dyDescent="0.3">
       <c r="C78" s="28" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="79" spans="1:22" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:22" ht="100.8" x14ac:dyDescent="0.3">
       <c r="B79" s="36" t="s">
         <v>201</v>
       </c>
@@ -4587,7 +4601,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="80" spans="1:22" ht="87" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:22" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A80" s="1" t="s">
         <v>197</v>
       </c>
@@ -4598,7 +4612,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="81" spans="1:22" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:22" ht="72" x14ac:dyDescent="0.3">
       <c r="A81" s="1" t="s">
         <v>196</v>
       </c>
@@ -4606,7 +4620,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="82" spans="1:22" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:22" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A82" s="1" t="s">
         <v>198</v>
       </c>
@@ -4614,10 +4628,10 @@
         <v>200</v>
       </c>
     </row>
-    <row r="83" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:22" x14ac:dyDescent="0.3">
       <c r="C83" s="35"/>
     </row>
-    <row r="84" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A84" s="3"/>
       <c r="B84" s="5"/>
       <c r="C84" s="6"/>
@@ -4636,7 +4650,7 @@
       <c r="S84" s="5"/>
       <c r="U84" s="5"/>
     </row>
-    <row r="85" spans="1:22" ht="29" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:22" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A85" s="1" t="s">
         <v>119</v>
       </c>
@@ -4650,17 +4664,17 @@
       <c r="U85" s="1"/>
       <c r="V85" s="2"/>
     </row>
-    <row r="86" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A86" s="11" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="87" spans="1:22" ht="29" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:22" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C87" s="28" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="88" spans="1:22" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:22" ht="72" x14ac:dyDescent="0.3">
       <c r="A88" s="2" t="s">
         <v>142</v>
       </c>
@@ -4668,27 +4682,27 @@
         <v>141</v>
       </c>
     </row>
-    <row r="89" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A89" s="12" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="90" spans="1:22" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:22" ht="43.2" x14ac:dyDescent="0.3">
       <c r="C90" s="28" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="91" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A91" s="12" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="92" spans="1:22" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:22" ht="100.8" x14ac:dyDescent="0.3">
       <c r="C92" s="28" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="94" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A94" s="3"/>
       <c r="B94" s="5"/>
       <c r="C94" s="6"/>
@@ -4707,7 +4721,7 @@
       <c r="S94" s="5"/>
       <c r="U94" s="5"/>
     </row>
-    <row r="95" spans="1:22" ht="29" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:22" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A95" s="1" t="s">
         <v>125</v>
       </c>
@@ -4721,7 +4735,7 @@
       <c r="U95" s="1"/>
       <c r="V95" s="2"/>
     </row>
-    <row r="98" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A98" s="3"/>
       <c r="B98" s="5"/>
       <c r="C98" s="6"/>
@@ -4740,7 +4754,7 @@
       <c r="S98" s="5"/>
       <c r="U98" s="5"/>
     </row>
-    <row r="99" spans="1:22" ht="29" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:22" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A99" s="1" t="s">
         <v>128</v>
       </c>
@@ -4754,17 +4768,17 @@
       <c r="U99" s="1"/>
       <c r="V99" s="2"/>
     </row>
-    <row r="100" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A100" s="11" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="101" spans="1:22" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:22" ht="158.4" x14ac:dyDescent="0.3">
       <c r="B101" s="28" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="103" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A103" s="3"/>
       <c r="B103" s="5"/>
       <c r="C103" s="6"/>
@@ -4783,7 +4797,7 @@
       <c r="S103" s="5"/>
       <c r="U103" s="5"/>
     </row>
-    <row r="104" spans="1:22" ht="29" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:22" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A104" s="1" t="s">
         <v>131</v>
       </c>
@@ -4797,37 +4811,37 @@
       <c r="U104" s="1"/>
       <c r="V104" s="2"/>
     </row>
-    <row r="105" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A105" s="11" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="106" spans="1:22" ht="29" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:22" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C106" s="28" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="107" spans="1:22" ht="29" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:22" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C107" s="28" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="108" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A108" s="11" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="109" spans="1:22" ht="29" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:22" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C109" s="28" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="110" spans="1:22" ht="29" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:22" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C110" s="28" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="112" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A112" s="3"/>
       <c r="B112" s="5"/>
       <c r="C112" s="6"/>
@@ -4846,7 +4860,7 @@
       <c r="S112" s="5"/>
       <c r="U112" s="5"/>
     </row>
-    <row r="113" spans="1:22" ht="29" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:22" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A113" s="1" t="s">
         <v>132</v>
       </c>
@@ -4860,12 +4874,12 @@
       <c r="U113" s="1"/>
       <c r="V113" s="2"/>
     </row>
-    <row r="114" spans="1:22" ht="29" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:22" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A114" s="30" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="115" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:22" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B115" s="2" t="s">
         <v>157</v>
       </c>
@@ -4873,7 +4887,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="116" spans="1:22" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:22" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B116" s="28" t="s">
         <v>160</v>
       </c>
@@ -4881,17 +4895,17 @@
         <v>159</v>
       </c>
     </row>
-    <row r="117" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A117" s="11" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="118" spans="1:22" ht="29" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:22" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C118" s="28" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="119" spans="1:22" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:22" ht="72" x14ac:dyDescent="0.3">
       <c r="B119" s="28" t="s">
         <v>163</v>
       </c>
@@ -4899,7 +4913,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="121" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A121" s="3"/>
       <c r="B121" s="5"/>
       <c r="C121" s="6"/>
@@ -4918,7 +4932,7 @@
       <c r="S121" s="5"/>
       <c r="U121" s="5"/>
     </row>
-    <row r="122" spans="1:22" ht="29" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:22" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A122" s="1" t="s">
         <v>164</v>
       </c>
@@ -4929,30 +4943,30 @@
       <c r="U122" s="1"/>
       <c r="V122" s="2"/>
     </row>
-    <row r="123" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A123" s="11" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="124" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A124" s="2"/>
       <c r="C124" s="32" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="125" spans="1:22" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:22" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A125" s="2"/>
       <c r="C125" s="32" t="s">
         <v>176</v>
       </c>
     </row>
-    <row r="126" spans="1:22" ht="29" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:22" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A126" s="2"/>
       <c r="C126" s="32" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="127" spans="1:22" ht="29" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:22" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A127" s="2"/>
       <c r="B127" s="15" t="s">
         <v>169</v>
@@ -4961,12 +4975,12 @@
         <v>168</v>
       </c>
     </row>
-    <row r="128" spans="1:22" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:22" ht="158.4" x14ac:dyDescent="0.3">
       <c r="C128" s="32" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="129" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:22" x14ac:dyDescent="0.3">
       <c r="B129" s="33" t="s">
         <v>170</v>
       </c>
@@ -4977,12 +4991,12 @@
         <v>165</v>
       </c>
     </row>
-    <row r="130" spans="1:22" ht="188.5" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:22" ht="187.2" x14ac:dyDescent="0.3">
       <c r="C130" s="32" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="131" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:22" x14ac:dyDescent="0.3">
       <c r="B131" s="34" t="s">
         <v>171</v>
       </c>
@@ -4993,12 +5007,12 @@
         <v>174</v>
       </c>
     </row>
-    <row r="132" spans="1:22" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:22" ht="72" x14ac:dyDescent="0.3">
       <c r="C132" s="32" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="133" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A133" s="3"/>
       <c r="B133" s="5"/>
       <c r="C133" s="6"/>
@@ -5017,7 +5031,7 @@
       <c r="S133" s="5"/>
       <c r="U133" s="5"/>
     </row>
-    <row r="134" spans="1:22" ht="29" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:22" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A134" s="1" t="s">
         <v>181</v>
       </c>
@@ -5028,27 +5042,27 @@
       <c r="U134" s="1"/>
       <c r="V134" s="2"/>
     </row>
-    <row r="135" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A135" s="11" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="136" spans="1:22" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:22" ht="43.2" x14ac:dyDescent="0.3">
       <c r="C136" s="32" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="137" spans="1:22" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:22" ht="72" x14ac:dyDescent="0.3">
       <c r="C137" s="32" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="138" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:22" x14ac:dyDescent="0.3">
       <c r="C138" s="32" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="139" spans="1:22" ht="87" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:22" ht="86.4" x14ac:dyDescent="0.3">
       <c r="B139" s="2" t="s">
         <v>191</v>
       </c>
@@ -5059,7 +5073,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="140" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:22" x14ac:dyDescent="0.3">
       <c r="B140" s="2" t="s">
         <v>190</v>
       </c>
@@ -5067,7 +5081,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="141" spans="1:22" ht="58" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:22" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B141" s="2" t="s">
         <v>192</v>
       </c>
@@ -5076,7 +5090,7 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="9" type="noConversion"/>
+  <phoneticPr fontId="10" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="10" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
   <drawing r:id="rId2"/>

</xml_diff>